<commit_message>
Update 5월 회비 데이터 and fix dynamic forecast labels
- 사군자.xlsx: 5월 회비 납부 내역 업데이트
- dashboard.py: Balance Forecast 월 계산을 마지막 실제 데이터 월 기준으로 동적 처리

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/사군자.xlsx
+++ b/data/사군자.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\sajunja-finance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01265D9-D5D8-4830-9D85-D8C99E1F3D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{006F5575-35B0-4C55-9D58-03D7EC3A5D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="165">
   <si>
     <t>No</t>
   </si>
@@ -521,6 +521,30 @@
   </si>
   <si>
     <t>한해 개업 화환</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>박승현 축의금</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>강명신 축의금</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>강연비</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>옥지엽, 공간대여</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>옥지엽, 강연비</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>옥지엽, 음식값</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -920,7 +944,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1220,9 +1244,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2401,13 +2422,13 @@
       <c r="B1" s="18"/>
       <c r="C1" s="19" t="str">
         <f ca="1">참고!$E$5</f>
-        <v>26년 3월</v>
+        <v>26년 4월</v>
       </c>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
       <c r="F1" s="19" t="str">
         <f ca="1">참고!$D$5</f>
-        <v>26년 4월</v>
+        <v>26년 5월</v>
       </c>
       <c r="G1" s="18"/>
       <c r="H1" s="18"/>
@@ -2454,19 +2475,19 @@
       <c r="C4" s="31"/>
       <c r="D4" s="35">
         <f ca="1">SUM(C5:C7)</f>
-        <v>2050568</v>
+        <v>2100380</v>
       </c>
       <c r="E4" s="40"/>
       <c r="F4" s="36"/>
       <c r="G4" s="37">
         <f ca="1">SUM(F5:F7)</f>
-        <v>2100380</v>
+        <v>2100425</v>
       </c>
       <c r="H4" s="40"/>
       <c r="I4" s="37"/>
       <c r="J4" s="37">
         <f>SUM(I5:I7)</f>
-        <v>40080698</v>
+        <v>42481123</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2476,7 +2497,7 @@
       <c r="B5" s="41"/>
       <c r="C5" s="29">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A5,원장!$A:$A,회비입출내역!$C$1)</f>
-        <v>1900000</v>
+        <v>2100000</v>
       </c>
       <c r="D5" s="30"/>
       <c r="E5" s="41"/>
@@ -2488,7 +2509,7 @@
       <c r="H5" s="41"/>
       <c r="I5" s="20">
         <f>SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A5)</f>
-        <v>39800000</v>
+        <v>42200000</v>
       </c>
       <c r="J5" s="21"/>
     </row>
@@ -2499,7 +2520,7 @@
       <c r="B6" s="41"/>
       <c r="C6" s="29">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A6,원장!$A:$A,회비입출내역!$C$1)</f>
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="41"/>
@@ -2522,19 +2543,19 @@
       <c r="B7" s="41"/>
       <c r="C7" s="29">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A7,원장!$A:$A,회비입출내역!$C$1)</f>
-        <v>568</v>
+        <v>380</v>
       </c>
       <c r="D7" s="30"/>
       <c r="E7" s="41"/>
       <c r="F7" s="28">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A7,원장!$A:$A,회비입출내역!$F$1)</f>
-        <v>380</v>
+        <v>425</v>
       </c>
       <c r="G7" s="21"/>
       <c r="H7" s="41"/>
       <c r="I7" s="20">
         <f>SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A7)</f>
-        <v>10698</v>
+        <v>11123</v>
       </c>
       <c r="J7" s="21"/>
     </row>
@@ -2558,19 +2579,19 @@
       <c r="C9" s="27"/>
       <c r="D9" s="35">
         <f ca="1">SUM(C10:C15)</f>
-        <v>-630000</v>
+        <v>-777550</v>
       </c>
       <c r="E9" s="40"/>
       <c r="F9" s="38"/>
       <c r="G9" s="37">
         <f ca="1">SUM(F10:F15)</f>
-        <v>-777550</v>
+        <v>-3149400</v>
       </c>
       <c r="H9" s="40"/>
       <c r="I9" s="39"/>
       <c r="J9" s="37">
         <f>SUM(I10:I15)</f>
-        <v>-33047950</v>
+        <v>-36197350</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2580,19 +2601,19 @@
       <c r="B10" s="46"/>
       <c r="C10" s="20">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A10,원장!$A:$A,회비입출내역!$C$1)</f>
-        <v>-630000</v>
+        <v>-728550</v>
       </c>
       <c r="D10" s="20"/>
       <c r="E10" s="42"/>
       <c r="F10" s="28">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A10,원장!$A:$A,회비입출내역!$F$1)</f>
-        <v>-728550</v>
+        <v>-285000</v>
       </c>
       <c r="G10" s="20"/>
       <c r="H10" s="42"/>
       <c r="I10" s="20">
         <f>SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A10)</f>
-        <v>-23084800</v>
+        <v>-23369800</v>
       </c>
       <c r="J10" s="20"/>
     </row>
@@ -2609,13 +2630,13 @@
       <c r="E11" s="42"/>
       <c r="F11" s="28">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A11,원장!$A:$A,회비입출내역!$F$1)</f>
-        <v>0</v>
+        <v>-864400</v>
       </c>
       <c r="G11" s="20"/>
       <c r="H11" s="42"/>
       <c r="I11" s="20">
         <f>SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A11)</f>
-        <v>-1870000</v>
+        <v>-2734400</v>
       </c>
       <c r="J11" s="20"/>
     </row>
@@ -2626,19 +2647,19 @@
       <c r="B12" s="43"/>
       <c r="C12" s="29">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A12,원장!$A:$A,회비입출내역!$C$1)</f>
-        <v>0</v>
+        <v>-49000</v>
       </c>
       <c r="D12" s="22"/>
       <c r="E12" s="43"/>
       <c r="F12" s="28">
         <f ca="1">SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A12,원장!$A:$A,회비입출내역!$F$1)</f>
-        <v>-49000</v>
+        <v>-2000000</v>
       </c>
       <c r="G12" s="22"/>
       <c r="H12" s="43"/>
       <c r="I12" s="20">
         <f>SUMIFS(원장!$H:$H,원장!$E:$E,회비입출내역!$A12)</f>
-        <v>-5168500</v>
+        <v>-7168500</v>
       </c>
       <c r="J12" s="22"/>
     </row>
@@ -2685,19 +2706,19 @@
       <c r="C15" s="27"/>
       <c r="D15" s="35">
         <f ca="1">SUM(D4:D13)</f>
-        <v>1420568</v>
+        <v>1322830</v>
       </c>
       <c r="E15" s="40"/>
       <c r="F15" s="38"/>
       <c r="G15" s="37">
         <f ca="1">SUM(G4:G13)</f>
-        <v>1322830</v>
+        <v>-1048975</v>
       </c>
       <c r="H15" s="40"/>
       <c r="I15" s="39"/>
       <c r="J15" s="37">
         <f>SUM(J4:J13)</f>
-        <v>7032748</v>
+        <v>6283773</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2713,7 +2734,7 @@
         <v>155</v>
       </c>
       <c r="J16" s="24">
-        <v>7032748</v>
+        <v>6283773</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -2940,83 +2961,83 @@
       </c>
       <c r="B3" s="6">
         <f t="shared" ref="B3:X3" si="0">SUM(B4:B101)</f>
-        <v>2300000</v>
+        <v>2500000</v>
       </c>
       <c r="C3" s="6">
         <f t="shared" si="0"/>
-        <v>2200000</v>
+        <v>2300000</v>
       </c>
       <c r="D3" s="6">
         <f t="shared" si="0"/>
-        <v>2300000</v>
+        <v>2400000</v>
       </c>
       <c r="E3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2500000</v>
       </c>
       <c r="F3" s="6">
         <f t="shared" si="0"/>
-        <v>2300000</v>
+        <v>2500000</v>
       </c>
       <c r="G3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2500000</v>
       </c>
       <c r="H3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2500000</v>
       </c>
       <c r="I3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2500000</v>
       </c>
       <c r="J3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2500000</v>
       </c>
       <c r="K3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2600000</v>
       </c>
       <c r="L3" s="6">
         <f t="shared" si="0"/>
-        <v>2300000</v>
+        <v>2500000</v>
       </c>
       <c r="M3" s="6">
         <f t="shared" si="0"/>
-        <v>2400000</v>
+        <v>2500000</v>
       </c>
       <c r="N3" s="6">
         <f t="shared" si="0"/>
-        <v>1800000</v>
+        <v>1900000</v>
       </c>
       <c r="O3" s="6">
         <f t="shared" si="0"/>
-        <v>1800000</v>
+        <v>1900000</v>
       </c>
       <c r="P3" s="6">
         <f t="shared" si="0"/>
-        <v>1800000</v>
+        <v>1900000</v>
       </c>
       <c r="Q3" s="6">
         <f t="shared" si="0"/>
-        <v>1600000</v>
+        <v>1700000</v>
       </c>
       <c r="R3" s="6">
         <f t="shared" si="0"/>
-        <v>1100000</v>
+        <v>1200000</v>
       </c>
       <c r="S3" s="6">
         <f t="shared" si="0"/>
-        <v>600000</v>
+        <v>700000</v>
       </c>
       <c r="T3" s="6">
         <f t="shared" si="0"/>
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="U3" s="6">
         <f t="shared" si="0"/>
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="V3" s="6">
         <f t="shared" si="0"/>
@@ -3032,7 +3053,7 @@
       </c>
       <c r="Y3" s="6">
         <f t="shared" ref="Y3:Y34" si="1">SUM(B3:X3)</f>
-        <v>39800000</v>
+        <v>42200000</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
@@ -4537,22 +4558,28 @@
       <c r="A27" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="101"/>
+      <c r="B27" s="25">
+        <v>100000</v>
+      </c>
       <c r="C27" s="25">
         <v>100000</v>
       </c>
-      <c r="D27" s="101"/>
+      <c r="D27" s="25">
+        <v>100000</v>
+      </c>
       <c r="E27" s="25">
         <v>100000</v>
       </c>
-      <c r="F27" s="69"/>
+      <c r="F27" s="25">
+        <v>100000</v>
+      </c>
       <c r="G27" s="25">
         <v>100000</v>
       </c>
       <c r="H27" s="25">
         <v>100000</v>
       </c>
-      <c r="I27" s="100">
+      <c r="I27" s="25">
         <v>100000</v>
       </c>
       <c r="J27" s="25">
@@ -4561,7 +4588,9 @@
       <c r="K27" s="25">
         <v>100000</v>
       </c>
-      <c r="L27" s="101"/>
+      <c r="L27" s="25">
+        <v>100000</v>
+      </c>
       <c r="M27" s="25">
         <v>100000</v>
       </c>
@@ -4574,7 +4603,9 @@
       <c r="P27" s="25">
         <v>100000</v>
       </c>
-      <c r="Q27" s="101"/>
+      <c r="Q27" s="25">
+        <v>100000</v>
+      </c>
       <c r="R27" s="100">
         <v>100000</v>
       </c>
@@ -4594,41 +4625,75 @@
       <c r="X27" s="4"/>
       <c r="Y27" s="6">
         <f t="shared" si="1"/>
-        <v>1600000</v>
+        <v>2100000</v>
       </c>
     </row>
     <row r="28" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="26"/>
-      <c r="H28" s="26"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
+      <c r="B28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="C28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="D28" s="69"/>
+      <c r="E28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="F28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="G28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="H28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="I28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="J28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="K28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="L28" s="25">
+        <v>100000</v>
+      </c>
       <c r="M28" s="25">
         <v>100000</v>
       </c>
-      <c r="N28" s="26"/>
-      <c r="O28" s="26"/>
-      <c r="P28" s="26"/>
-      <c r="Q28" s="26"/>
-      <c r="R28" s="26"/>
-      <c r="S28" s="26"/>
-      <c r="T28" s="26"/>
-      <c r="U28" s="26"/>
-      <c r="V28" s="26"/>
+      <c r="N28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="O28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="P28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="Q28" s="69"/>
+      <c r="R28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="S28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="T28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="U28" s="25">
+        <v>100000</v>
+      </c>
+      <c r="V28" s="69"/>
       <c r="W28" s="4"/>
       <c r="X28" s="4"/>
       <c r="Y28" s="6">
         <f t="shared" si="1"/>
-        <v>100000</v>
+        <v>1800000</v>
       </c>
     </row>
     <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4644,9 +4709,13 @@
       <c r="H29" s="26"/>
       <c r="I29" s="26"/>
       <c r="J29" s="26"/>
-      <c r="K29" s="26"/>
+      <c r="K29" s="25">
+        <v>100000</v>
+      </c>
       <c r="L29" s="26"/>
-      <c r="M29" s="26"/>
+      <c r="M29" s="25">
+        <v>100000</v>
+      </c>
       <c r="N29" s="26"/>
       <c r="O29" s="26"/>
       <c r="P29" s="26"/>
@@ -4660,7 +4729,7 @@
       <c r="X29" s="4"/>
       <c r="Y29" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="30" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4831,7 +4900,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K109"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.25" style="99" customWidth="1"/>
@@ -6851,7 +6920,7 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" s="10" t="str">
-        <f t="shared" ref="A67:A102" si="4">RIGHT(YEAR(C67),2)&amp;"년 "&amp;MONTH(C67)&amp;"월"</f>
+        <f t="shared" ref="A67:A107" si="4">RIGHT(YEAR(C67),2)&amp;"년 "&amp;MONTH(C67)&amp;"월"</f>
         <v>25년 9월</v>
       </c>
       <c r="B67" s="10" t="str">
@@ -6872,7 +6941,7 @@
       </c>
       <c r="G67" s="15"/>
       <c r="H67" s="17">
-        <f t="shared" ref="H67:H102" si="5">G67-F67</f>
+        <f t="shared" ref="H67:H98" si="5">G67-F67</f>
         <v>-508770</v>
       </c>
       <c r="I67" s="16" t="s">
@@ -7869,7 +7938,7 @@
       </c>
       <c r="G100" s="15"/>
       <c r="H100" s="17">
-        <f t="shared" ref="H100:H101" si="9">G100-F100</f>
+        <f t="shared" ref="H100:H103" si="9">G100-F100</f>
         <v>-361900</v>
       </c>
       <c r="I100" s="16" t="s">
@@ -7927,10 +7996,11 @@
       <c r="F102" s="15"/>
       <c r="G102" s="15">
         <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A102)</f>
-        <v>1600000</v>
+        <v>2100000</v>
       </c>
       <c r="H102" s="17">
-        <v>1600000</v>
+        <f t="shared" si="9"/>
+        <v>2100000</v>
       </c>
       <c r="I102" s="16" t="s">
         <v>89</v>
@@ -7938,201 +8008,196 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" s="10" t="str">
-        <f t="shared" ref="A103:A109" si="10">RIGHT(YEAR(C103),2)&amp;"년 "&amp;MONTH(C103)&amp;"월"</f>
-        <v>26년 6월</v>
+        <f t="shared" ref="A103" si="10">RIGHT(YEAR(C103),2)&amp;"년 "&amp;MONTH(C103)&amp;"월"</f>
+        <v>26년 5월</v>
       </c>
       <c r="B103" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C103,2),참조!$A$1:$B$10,2,)</f>
-        <v>월</v>
+        <v>일</v>
       </c>
       <c r="C103" s="14">
-        <v>46174</v>
+        <v>46173</v>
       </c>
       <c r="D103" s="14" t="s">
         <v>88</v>
       </c>
       <c r="E103" s="14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F103" s="15"/>
       <c r="G103" s="15">
-        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A103)</f>
-        <v>100000</v>
+        <v>425</v>
       </c>
       <c r="H103" s="17">
-        <f t="shared" ref="H103:H109" si="11">G103-F103</f>
-        <v>100000</v>
+        <f t="shared" si="9"/>
+        <v>425</v>
       </c>
       <c r="I103" s="16" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" s="10" t="str">
-        <f t="shared" si="10"/>
-        <v>26년 7월</v>
+        <f t="shared" si="4"/>
+        <v>26년 5월</v>
       </c>
       <c r="B104" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C104,2),참조!$A$1:$B$10,2,)</f>
-        <v>수</v>
+        <v>일</v>
       </c>
       <c r="C104" s="14">
-        <v>46204</v>
+        <v>46159</v>
       </c>
       <c r="D104" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E104" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F104" s="15"/>
-      <c r="G104" s="15">
-        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A104)</f>
-        <v>0</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="F104" s="15">
+        <f>875000-590000</f>
+        <v>285000</v>
+      </c>
+      <c r="G104" s="15"/>
       <c r="H104" s="17">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <f t="shared" ref="H104" si="11">G104-F104</f>
+        <v>-285000</v>
       </c>
       <c r="I104" s="16" t="s">
-        <v>89</v>
+        <v>162</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105" s="10" t="str">
-        <f t="shared" si="10"/>
-        <v>26년 8월</v>
+        <f t="shared" ref="A105" si="12">RIGHT(YEAR(C105),2)&amp;"년 "&amp;MONTH(C105)&amp;"월"</f>
+        <v>26년 5월</v>
       </c>
       <c r="B105" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C105,2),참조!$A$1:$B$10,2,)</f>
-        <v>토</v>
+        <v>일</v>
       </c>
       <c r="C105" s="14">
-        <v>46235</v>
+        <v>46159</v>
       </c>
       <c r="D105" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E105" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F105" s="15"/>
-      <c r="G105" s="15">
-        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A105)</f>
-        <v>0</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="F105" s="15">
+        <v>590000</v>
+      </c>
+      <c r="G105" s="15"/>
       <c r="H105" s="17">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <f t="shared" ref="H105" si="13">G105-F105</f>
+        <v>-590000</v>
       </c>
       <c r="I105" s="16" t="s">
-        <v>89</v>
+        <v>163</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" s="10" t="str">
-        <f t="shared" si="10"/>
-        <v>26년 9월</v>
+        <f t="shared" ref="A106" si="14">RIGHT(YEAR(C106),2)&amp;"년 "&amp;MONTH(C106)&amp;"월"</f>
+        <v>26년 5월</v>
       </c>
       <c r="B106" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C106,2),참조!$A$1:$B$10,2,)</f>
-        <v>화</v>
+        <v>일</v>
       </c>
       <c r="C106" s="14">
-        <v>46266</v>
+        <v>46159</v>
       </c>
       <c r="D106" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E106" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F106" s="15"/>
-      <c r="G106" s="15">
-        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A106)</f>
-        <v>0</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="F106" s="15">
+        <v>274400</v>
+      </c>
+      <c r="G106" s="15"/>
       <c r="H106" s="17">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <f t="shared" ref="H106" si="15">G106-F106</f>
+        <v>-274400</v>
       </c>
       <c r="I106" s="16" t="s">
-        <v>89</v>
+        <v>164</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="str">
-        <f t="shared" si="10"/>
-        <v>26년 10월</v>
+        <f t="shared" si="4"/>
+        <v>26년 5월</v>
       </c>
       <c r="B107" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C107,2),참조!$A$1:$B$10,2,)</f>
-        <v>목</v>
+        <v>일</v>
       </c>
       <c r="C107" s="14">
-        <v>46296</v>
+        <v>46159</v>
       </c>
       <c r="D107" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E107" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F107" s="15"/>
-      <c r="G107" s="15">
-        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A107)</f>
-        <v>0</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="F107" s="15">
+        <v>1000000</v>
+      </c>
+      <c r="G107" s="15"/>
       <c r="H107" s="17">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <f t="shared" ref="H107" si="16">G107-F107</f>
+        <v>-1000000</v>
       </c>
       <c r="I107" s="16" t="s">
-        <v>89</v>
+        <v>160</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" s="10" t="str">
-        <f t="shared" si="10"/>
-        <v>26년 11월</v>
+        <f t="shared" ref="A108" si="17">RIGHT(YEAR(C108),2)&amp;"년 "&amp;MONTH(C108)&amp;"월"</f>
+        <v>26년 5월</v>
       </c>
       <c r="B108" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C108,2),참조!$A$1:$B$10,2,)</f>
         <v>일</v>
       </c>
       <c r="C108" s="14">
-        <v>46327</v>
+        <v>46173</v>
       </c>
       <c r="D108" s="14" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E108" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F108" s="15"/>
-      <c r="G108" s="15">
-        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A108)</f>
-        <v>0</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="F108" s="15">
+        <v>1000000</v>
+      </c>
+      <c r="G108" s="15"/>
       <c r="H108" s="17">
-        <f t="shared" si="11"/>
-        <v>0</v>
+        <f t="shared" ref="H108" si="18">G108-F108</f>
+        <v>-1000000</v>
       </c>
       <c r="I108" s="16" t="s">
-        <v>89</v>
+        <v>159</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" s="10" t="str">
-        <f t="shared" si="10"/>
-        <v>26년 12월</v>
+        <f t="shared" ref="A109:A115" si="19">RIGHT(YEAR(C109),2)&amp;"년 "&amp;MONTH(C109)&amp;"월"</f>
+        <v>26년 6월</v>
       </c>
       <c r="B109" s="10" t="str">
         <f>VLOOKUP(WEEKDAY(C109,2),참조!$A$1:$B$10,2,)</f>
-        <v>화</v>
+        <v>월</v>
       </c>
       <c r="C109" s="14">
-        <v>46357</v>
+        <v>46174</v>
       </c>
       <c r="D109" s="14" t="s">
         <v>88</v>
@@ -8143,13 +8208,199 @@
       <c r="F109" s="15"/>
       <c r="G109" s="15">
         <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A109)</f>
+        <v>1800000</v>
+      </c>
+      <c r="H109" s="17">
+        <f t="shared" ref="H109:H115" si="20">G109-F109</f>
+        <v>1800000</v>
+      </c>
+      <c r="I109" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A110" s="10" t="str">
+        <f t="shared" si="19"/>
+        <v>26년 7월</v>
+      </c>
+      <c r="B110" s="10" t="str">
+        <f>VLOOKUP(WEEKDAY(C110,2),참조!$A$1:$B$10,2,)</f>
+        <v>수</v>
+      </c>
+      <c r="C110" s="14">
+        <v>46204</v>
+      </c>
+      <c r="D110" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E110" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F110" s="15"/>
+      <c r="G110" s="15">
+        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A110)</f>
+        <v>200000</v>
+      </c>
+      <c r="H110" s="17">
+        <f t="shared" si="20"/>
+        <v>200000</v>
+      </c>
+      <c r="I110" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A111" s="10" t="str">
+        <f t="shared" si="19"/>
+        <v>26년 8월</v>
+      </c>
+      <c r="B111" s="10" t="str">
+        <f>VLOOKUP(WEEKDAY(C111,2),참조!$A$1:$B$10,2,)</f>
+        <v>토</v>
+      </c>
+      <c r="C111" s="14">
+        <v>46235</v>
+      </c>
+      <c r="D111" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E111" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F111" s="15"/>
+      <c r="G111" s="15">
+        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A111)</f>
         <v>0</v>
       </c>
-      <c r="H109" s="17">
-        <f t="shared" si="11"/>
+      <c r="H111" s="17">
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="I109" s="16" t="s">
+      <c r="I111" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A112" s="10" t="str">
+        <f t="shared" si="19"/>
+        <v>26년 9월</v>
+      </c>
+      <c r="B112" s="10" t="str">
+        <f>VLOOKUP(WEEKDAY(C112,2),참조!$A$1:$B$10,2,)</f>
+        <v>화</v>
+      </c>
+      <c r="C112" s="14">
+        <v>46266</v>
+      </c>
+      <c r="D112" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E112" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F112" s="15"/>
+      <c r="G112" s="15">
+        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A112)</f>
+        <v>0</v>
+      </c>
+      <c r="H112" s="17">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="I112" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A113" s="10" t="str">
+        <f t="shared" si="19"/>
+        <v>26년 10월</v>
+      </c>
+      <c r="B113" s="10" t="str">
+        <f>VLOOKUP(WEEKDAY(C113,2),참조!$A$1:$B$10,2,)</f>
+        <v>목</v>
+      </c>
+      <c r="C113" s="14">
+        <v>46296</v>
+      </c>
+      <c r="D113" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E113" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F113" s="15"/>
+      <c r="G113" s="15">
+        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A113)</f>
+        <v>0</v>
+      </c>
+      <c r="H113" s="17">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="I113" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A114" s="10" t="str">
+        <f t="shared" si="19"/>
+        <v>26년 11월</v>
+      </c>
+      <c r="B114" s="10" t="str">
+        <f>VLOOKUP(WEEKDAY(C114,2),참조!$A$1:$B$10,2,)</f>
+        <v>일</v>
+      </c>
+      <c r="C114" s="14">
+        <v>46327</v>
+      </c>
+      <c r="D114" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E114" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F114" s="15"/>
+      <c r="G114" s="15">
+        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A114)</f>
+        <v>0</v>
+      </c>
+      <c r="H114" s="17">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="I114" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A115" s="10" t="str">
+        <f t="shared" si="19"/>
+        <v>26년 12월</v>
+      </c>
+      <c r="B115" s="10" t="str">
+        <f>VLOOKUP(WEEKDAY(C115,2),참조!$A$1:$B$10,2,)</f>
+        <v>화</v>
+      </c>
+      <c r="C115" s="14">
+        <v>46357</v>
+      </c>
+      <c r="D115" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E115" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F115" s="15"/>
+      <c r="G115" s="15">
+        <f>SUMIFS(입금현황!$Y:$Y,입금현황!$A:$A,원장!$A115)</f>
+        <v>0</v>
+      </c>
+      <c r="H115" s="17">
+        <f t="shared" si="20"/>
+        <v>0</v>
+      </c>
+      <c r="I115" s="16" t="s">
         <v>89</v>
       </c>
     </row>
@@ -10043,7 +10294,7 @@
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="68">
         <f ca="1">TODAY()</f>
-        <v>46147</v>
+        <v>46176</v>
       </c>
       <c r="B1" s="67">
         <f ca="1">YEAR(A1)</f>
@@ -10051,55 +10302,55 @@
       </c>
       <c r="C1" s="67">
         <f ca="1">MONTH(A1)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" s="67">
         <f t="shared" ref="D1:O1" ca="1" si="0">IF(C1-1=0,12,C1-1)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="I1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O1" s="67">
         <f t="shared" ca="1" si="0"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
@@ -10125,101 +10376,101 @@
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D4" s="67" t="str">
         <f t="shared" ref="D4:O4" ca="1" si="1">D1&amp;"월"</f>
-        <v>4월</v>
+        <v>5월</v>
       </c>
       <c r="E4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>3월</v>
+        <v>4월</v>
       </c>
       <c r="F4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>2월</v>
+        <v>3월</v>
       </c>
       <c r="G4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>1월</v>
+        <v>2월</v>
       </c>
       <c r="H4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>12월</v>
+        <v>1월</v>
       </c>
       <c r="I4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>11월</v>
+        <v>12월</v>
       </c>
       <c r="J4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>10월</v>
+        <v>11월</v>
       </c>
       <c r="K4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>9월</v>
+        <v>10월</v>
       </c>
       <c r="L4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>8월</v>
+        <v>9월</v>
       </c>
       <c r="M4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>7월</v>
+        <v>8월</v>
       </c>
       <c r="N4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>6월</v>
+        <v>7월</v>
       </c>
       <c r="O4" s="67" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>5월</v>
+        <v>6월</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="D5" s="67" t="str">
         <f t="shared" ref="D5:O5" ca="1" si="2">IF(D1&gt;=$C$1,$C$3&amp;" "&amp;D4,$B$3&amp;" "&amp;D4)</f>
-        <v>26년 4월</v>
+        <v>26년 5월</v>
       </c>
       <c r="E5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>26년 3월</v>
+        <v>26년 4월</v>
       </c>
       <c r="F5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>26년 2월</v>
+        <v>26년 3월</v>
       </c>
       <c r="G5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>26년 1월</v>
+        <v>26년 2월</v>
       </c>
       <c r="H5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 12월</v>
+        <v>26년 1월</v>
       </c>
       <c r="I5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 11월</v>
+        <v>25년 12월</v>
       </c>
       <c r="J5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 10월</v>
+        <v>25년 11월</v>
       </c>
       <c r="K5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 9월</v>
+        <v>25년 10월</v>
       </c>
       <c r="L5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 8월</v>
+        <v>25년 9월</v>
       </c>
       <c r="M5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 7월</v>
+        <v>25년 8월</v>
       </c>
       <c r="N5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 6월</v>
+        <v>25년 7월</v>
       </c>
       <c r="O5" s="67" t="str">
         <f t="shared" ca="1" si="2"/>
-        <v>25년 5월</v>
+        <v>25년 6월</v>
       </c>
     </row>
   </sheetData>
@@ -10272,11 +10523,11 @@
       </c>
       <c r="F9" s="94" t="str">
         <f ca="1">회비입출내역!F1</f>
-        <v>26년 4월</v>
+        <v>26년 5월</v>
       </c>
       <c r="G9" s="81" t="str">
         <f ca="1">회비입출내역!$C$1</f>
-        <v>26년 3월</v>
+        <v>26년 4월</v>
       </c>
       <c r="H9" s="81" t="str">
         <f>증감분석!B5</f>
@@ -10302,11 +10553,11 @@
       </c>
       <c r="F10" s="95">
         <f ca="1">회비입출내역!$G$4</f>
-        <v>2100380</v>
+        <v>2100425</v>
       </c>
       <c r="G10" s="82">
         <f ca="1">회비입출내역!$D$4</f>
-        <v>2050568</v>
+        <v>2100380</v>
       </c>
       <c r="H10" s="75">
         <f ca="1">증감분석!$G$5</f>
@@ -10322,7 +10573,7 @@
       </c>
       <c r="K10" s="74">
         <f>회비입출내역!$J$4</f>
-        <v>40080698</v>
+        <v>42481123</v>
       </c>
       <c r="M10" s="89"/>
     </row>
@@ -10333,11 +10584,11 @@
       </c>
       <c r="F11" s="96">
         <f ca="1">회비입출내역!$G$9</f>
-        <v>-777550</v>
+        <v>-3149400</v>
       </c>
       <c r="G11" s="83">
         <f ca="1">회비입출내역!$D$9</f>
-        <v>-630000</v>
+        <v>-777550</v>
       </c>
       <c r="H11" s="60">
         <f ca="1">증감분석!$L$5</f>
@@ -10353,7 +10604,7 @@
       </c>
       <c r="K11" s="76">
         <f>회비입출내역!$J$9</f>
-        <v>-33047950</v>
+        <v>-36197350</v>
       </c>
       <c r="M11" s="89"/>
     </row>
@@ -10364,11 +10615,11 @@
       </c>
       <c r="F12" s="97">
         <f t="shared" ref="F12:K12" ca="1" si="0">SUM(F10:F11)</f>
-        <v>1322830</v>
+        <v>-1048975</v>
       </c>
       <c r="G12" s="63">
         <f t="shared" ca="1" si="0"/>
-        <v>1420568</v>
+        <v>1322830</v>
       </c>
       <c r="H12" s="63">
         <f t="shared" ca="1" si="0"/>
@@ -10384,7 +10635,7 @@
       </c>
       <c r="K12" s="60">
         <f t="shared" si="0"/>
-        <v>7032748</v>
+        <v>6283773</v>
       </c>
       <c r="M12" s="89"/>
     </row>

</xml_diff>